<commit_message>
Estonia 121/122: enumeración precisa de sectores (elaboración e implementación)
Sin cambio de puntaje (121=4, 122=4); se refina el "por qué" con los sectores nombrados
en el texto primario:
- ELABORACIÓN (121, VR p.8/12, PA p.6): Gobierno + privado (eraettevõtted, ITL,
  consorcios, parques científicos) + academia (universidades, Eesti Keele Instituut) +
  sociedad civil (vabaühendused) → Gob+3.
- IMPLEMENTACIÓN (122, VR p.12/33): Gobierno (juhtrühmad MKM + RIA + Statistikaamet +
  gobiernos locales + centros de competencia) + privado (erasektor, AIRE) + academia
  (universidades vía AIRE, Eesti Keele Instituut) + "väliste võtmepartnerite" / red de
  datos abierta → Gob+3 = 4 (estricto por sectores nombrados privado+academia: 3).

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/por_pais/Gobernanza_EE_Estonia_ILIA2026.xlsx
+++ b/data/paises_extra/por_pais/Gobernanza_EE_Estonia_ILIA2026.xlsx
@@ -1156,13 +1156,13 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Multistakeholder en la elaboración = Gob + sector privado (ITL, eraettevõtted, consorcios, teaduspargid) + academia (ülikoolid) + sociedad civil (vabaühendused). Valge raamat p.8/12 → Gob+3.  [confianza: ALTA]</t>
+          <t>Sectores en la ELABORACIÓN (VR p.8/12, PA p.6): GOBIERNO (MKM líder + Justiitsmin., HTM, Riigikantselei, todos los ministerios y agencias) + PRIVADO (eraettevõtted, asociación ITL, consorcios de empresas, teaduspargid) + ACADEMIA (ülikoolid, instituciones de educación/investigación, Eesti Keele Instituut) + SOCIEDAD CIVIL (vabaühendused). → Gob+3 = 4.  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>[oficial] https://knowledge4policy.ec.europa.eu/sites/default/files/estonia-ai-strategy-report.pdf
-[secundaria] https://regulations.ai/regulations/RAI-EE-NA-DAIWPXX-2024</t>
+          <t>[secundaria] https://regulations.ai/regulations/RAI-EE-NA-DAIWPXX-2024
+[secundaria] https://regulations.ai/regulations/RAI-EE-NA-ADAPKXX-2024</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Implementación vía juhtrühmad (MKM + asutused + 'avaliku sektori välised võtmepartnerid', p.12); áreas del AP: público, privado, academia → Gob+3.  [confianza: MEDIA-ALTA]</t>
+          <t>Sectores en la IMPLEMENTACIÓN (VR p.12/33): GOBIERNO (juhtrühmad liderados por MKM + ministerios + RIA + Statistikaamet + gobiernos locales + centros de competencia) + PRIVADO (erasektor; empresas vía AIRE) + ACADEMIA (universidades asociadas vía AIRE; Eesti Keele Instituut); las juhtrühmad suman 'avaliku sektori välised võtmepartnerid' y rinden cuentas al público vía 'andmete võrgustiku avatud kohtumine'. → Gob+3 = 4 (estricto por sectores nombrados privado+academia: Gob+2 = 3).  [confianza: MEDIA-ALTA]</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">

</xml_diff>